<commit_message>
subida documentos para repositorio actualizados
</commit_message>
<xml_diff>
--- a/Fase_2/Evidencias_Proyecto/Evidencia_Documentacion/Documentos_Scrum/Plantilla Historias Usuario con instructivo.xlsx
+++ b/Fase_2/Evidencias_Proyecto/Evidencia_Documentacion/Documentos_Scrum/Plantilla Historias Usuario con instructivo.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="qABYXyDv4XV1k9Hnc7UImvFDKBY+xEerPRlUdSn95mM="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="EIigcu6RhQp8KaEv8ZtUq0K+WJXP+6rMLZNTVaaBnsA="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="108">
   <si>
     <t>Historias de usuario y criterios de aceptación: Instructivo</t>
   </si>
@@ -62,22 +62,19 @@
     <t>Lo que el rol necesita lograr al ejecutar la acción. Este es el resultado de ejecutar la acción desde el punto de vista del rol. Este punto puede ser opcional, pues la historia puede documentarse sólo con la definición del rol y la acción (sin definir la consecuencia).</t>
   </si>
   <si>
-    <t>Enunciado de la historia</t>
-  </si>
-  <si>
     <t>Número (#) de escenario</t>
   </si>
   <si>
     <t>Número (ejemplo 1, 2, 3 ó 4), que identifica al escenario asociado a la historia.</t>
   </si>
   <si>
-    <t>Criterios de aceptación</t>
-  </si>
-  <si>
     <t>Criterio de aceptación (título)</t>
   </si>
   <si>
     <t>Describe el contexto del escenario que define un comportamiento. Por ejemplo, si se toma el ejemplo de búsquedas de productos por categoría, un posible ejemplo pudiera ser: Categoría sin productos asociados.</t>
+  </si>
+  <si>
+    <t>Enunciado de la historia</t>
   </si>
   <si>
     <t>Contexto</t>
@@ -92,13 +89,16 @@
     <t>Representa la acción que el usuario ejecuta, en el contexto definido para el escenario.</t>
   </si>
   <si>
-    <t>Criterio de aceptación (Título)</t>
-  </si>
-  <si>
     <t>Resultado / Comportamiento esperado</t>
   </si>
   <si>
     <t>Dado el contexto y la acción ejecutada por el usuario, la consecuencia es el comportamiento del sistema en esa situación.</t>
+  </si>
+  <si>
+    <t>Criterios de aceptación</t>
+  </si>
+  <si>
+    <t>Criterio de aceptación (Título)</t>
   </si>
   <si>
     <t>HCS-001</t>
@@ -659,22 +659,7 @@
     <t>Descargar planos actuales</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t xml:space="preserve">En caso que </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
-      </rPr>
-      <t>seleccione descargar los planos actuales</t>
-    </r>
+    <t>Cuando se selecciona descargar los planos actuales diseñados por el propio usuario</t>
   </si>
   <si>
     <r>
@@ -769,6 +754,81 @@
       <t>descargara el resumen de los materiales, precios y cantidades en formato PDF</t>
     </r>
   </si>
+  <si>
+    <t>HCS-005</t>
+  </si>
+  <si>
+    <t>Como un administrador del sistema</t>
+  </si>
+  <si>
+    <t>Necesito agregar, editar y eliminar materiales individuales en el catálogo</t>
+  </si>
+  <si>
+    <t>Con la finalidad de mantener la oferta del simulador actualizada con los nuevos insumos del mercado.</t>
+  </si>
+  <si>
+    <t>Inserción exitosa de material.</t>
+  </si>
+  <si>
+    <t>En caso que el administrador complete el formulario de un nuevo material con todos los datos obligatorios válidos.</t>
+  </si>
+  <si>
+    <t>Cuando presione el botón de guardar registro.</t>
+  </si>
+  <si>
+    <t>El sistema añadirá el ítem a la base de datos y este quedará disponible inmediatamente en el simulador de los usuarios.</t>
+  </si>
+  <si>
+    <t>Validación de campos obligatorios.</t>
+  </si>
+  <si>
+    <t>En caso que el administrador intente guardar un material dejando el precio, nombre o unidad de medida en blanco.</t>
+  </si>
+  <si>
+    <t>El sistema detendrá la acción, resaltará en rojo los campos faltantes y mostrará un mensaje indicando que se deben completar.</t>
+  </si>
+  <si>
+    <t>Eliminación de material registrado.</t>
+  </si>
+  <si>
+    <t>En caso que un material ya no esté a la venta pero haya sido utilizado en presupuestos históricos guardados por los usuarios</t>
+  </si>
+  <si>
+    <t>Cuando el administrador seleccione la opción de "Eliminar" sobre dicho material.</t>
+  </si>
+  <si>
+    <t>El sistema lo ocultará del catálogo para nuevas simulaciones (estado inactivo), pero mantendrá el registro interno para no alterar el historial de los proyectos antiguos.</t>
+  </si>
+  <si>
+    <t>HCS-006</t>
+  </si>
+  <si>
+    <t>Necesito configurar variables globales como el porcentaje de impuestos (ej. IVA) y costos base de despacho</t>
+  </si>
+  <si>
+    <t>Con la finalidad de que el cálculo final de los presupuestos de los usuarios cumpla con la normativa y logística vigente.</t>
+  </si>
+  <si>
+    <t>Ingreso porcentual positivo (+%)</t>
+  </si>
+  <si>
+    <t>En caso que se modifique el valor del impuesto aplicable para los materiales dispuestos a utilizarce dentro de plano automatico o manual de HouseCount.</t>
+  </si>
+  <si>
+    <t>El sistema utilizará el nuevo porcentaje para todos los presupuestos nuevos generados.</t>
+  </si>
+  <si>
+    <t>Ingreso de valores inválidos (-%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al momento de ingresar por error un valor de porcentaje negativo </t>
+  </si>
+  <si>
+    <t>Cuando se plantea generar una actualización a materiales ya establecidos</t>
+  </si>
+  <si>
+    <t>El sistema rechazará la acción, no guardará los cambios y mostrará una alerta de error, que destaca la equivocación señalada.</t>
+  </si>
 </sst>
 </file>
 
@@ -794,14 +854,14 @@
     </font>
     <font>
       <b/>
-      <sz val="28.0"/>
-      <color theme="1"/>
+      <sz val="16.0"/>
+      <color rgb="FF1F497D"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
-      <color rgb="FF1F497D"/>
+      <sz val="28.0"/>
+      <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -843,7 +903,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border/>
     <border>
       <left/>
@@ -935,11 +995,21 @@
       <top/>
       <bottom/>
     </border>
+    <border>
+      <left/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -991,6 +1061,11 @@
     <xf borderId="2" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
+    <xf borderId="10" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="2" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="11" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1210,8 +1285,8 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="1.43"/>
     <col customWidth="1" min="2" max="2" width="13.71"/>
-    <col customWidth="1" min="3" max="3" width="12.14"/>
-    <col customWidth="1" min="4" max="4" width="16.14"/>
+    <col customWidth="1" min="3" max="3" width="23.71"/>
+    <col customWidth="1" min="4" max="4" width="34.57"/>
     <col customWidth="1" min="5" max="5" width="21.57"/>
     <col customWidth="1" min="6" max="6" width="12.57"/>
     <col customWidth="1" min="7" max="7" width="21.29"/>
@@ -1223,7 +1298,7 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1"/>
@@ -1253,7 +1328,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="4"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1311,13 +1386,13 @@
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="7" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="9"/>
       <c r="G4" s="7" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="8"/>
@@ -1354,19 +1429,19 @@
         <v>10</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -1948,16 +2023,34 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
+      <c r="A21" s="23"/>
+      <c r="B21" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D21" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E21" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="G21" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="H21" s="21" t="s">
+        <v>88</v>
+      </c>
+      <c r="I21" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="J21" s="21" t="s">
+        <v>90</v>
+      </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
@@ -1976,16 +2069,26 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
+      <c r="A22" s="23"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="24">
+        <v>2.0</v>
+      </c>
+      <c r="G22" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="H22" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="I22" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="J22" s="21" t="s">
+        <v>93</v>
+      </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
@@ -2004,16 +2107,26 @@
       <c r="Z22" s="1"/>
     </row>
     <row r="23" ht="14.25" customHeight="1">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
+      <c r="A23" s="23"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="24">
+        <v>3.0</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="H23" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="I23" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="J23" s="21" t="s">
+        <v>97</v>
+      </c>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
@@ -2033,15 +2146,15 @@
     </row>
     <row r="24" ht="14.25" customHeight="1">
       <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+      <c r="J24" s="22"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
@@ -2060,16 +2173,34 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" ht="14.25" customHeight="1">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
+      <c r="A25" s="23"/>
+      <c r="B25" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="F25" s="20">
+        <v>1.0</v>
+      </c>
+      <c r="G25" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="H25" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="I25" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="J25" s="21" t="s">
+        <v>103</v>
+      </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
@@ -2088,16 +2219,26 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" ht="14.25" customHeight="1">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
+      <c r="A26" s="23"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="24">
+        <v>2.0</v>
+      </c>
+      <c r="G26" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="H26" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="I26" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="J26" s="21" t="s">
+        <v>107</v>
+      </c>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -2117,10 +2258,10 @@
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
@@ -29275,36 +29416,8 @@
       <c r="Y996" s="1"/>
       <c r="Z996" s="1"/>
     </row>
-    <row r="997" ht="14.25" customHeight="1">
-      <c r="A997" s="1"/>
-      <c r="B997" s="1"/>
-      <c r="C997" s="1"/>
-      <c r="D997" s="1"/>
-      <c r="E997" s="1"/>
-      <c r="F997" s="1"/>
-      <c r="G997" s="1"/>
-      <c r="H997" s="1"/>
-      <c r="I997" s="1"/>
-      <c r="J997" s="1"/>
-      <c r="K997" s="1"/>
-      <c r="L997" s="1"/>
-      <c r="M997" s="1"/>
-      <c r="N997" s="1"/>
-      <c r="O997" s="1"/>
-      <c r="P997" s="1"/>
-      <c r="Q997" s="1"/>
-      <c r="R997" s="1"/>
-      <c r="S997" s="1"/>
-      <c r="T997" s="1"/>
-      <c r="U997" s="1"/>
-      <c r="V997" s="1"/>
-      <c r="W997" s="1"/>
-      <c r="X997" s="1"/>
-      <c r="Y997" s="1"/>
-      <c r="Z997" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="26">
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="G4:J4"/>
     <mergeCell ref="B6:B8"/>
@@ -29313,8 +29426,6 @@
     <mergeCell ref="E6:E8"/>
     <mergeCell ref="B10:B13"/>
     <mergeCell ref="E10:E13"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
     <mergeCell ref="C10:C13"/>
     <mergeCell ref="D10:D13"/>
     <mergeCell ref="B15:B16"/>
@@ -29323,6 +29434,16 @@
     <mergeCell ref="E15:E16"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="E18:E19"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="E25:E26"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.7480314960629921" footer="0.0" header="0.0" left="0.7086614173228347" right="0.7086614173228347" top="0.7480314960629921"/>
@@ -29377,7 +29498,7 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="1"/>
-      <c r="B2" s="4"/>
+      <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -29594,10 +29715,10 @@
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" s="1"/>
       <c r="B9" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -29626,10 +29747,10 @@
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" s="1"/>
       <c r="B10" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -29658,10 +29779,10 @@
     <row r="11" ht="14.25" customHeight="1">
       <c r="A11" s="1"/>
       <c r="B11" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -29690,10 +29811,10 @@
     <row r="12" ht="14.25" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -29722,10 +29843,10 @@
     <row r="13" ht="14.25" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>

</xml_diff>